<commit_message>
chore: update SJPS progress card template data
</commit_message>
<xml_diff>
--- a/SJPS_progress card.xlsx
+++ b/SJPS_progress card.xlsx
@@ -890,7 +890,9 @@
       <c r="M13" s="7"/>
     </row>
     <row r="14" ht="24.75" customHeight="1">
-      <c r="A14" s="7"/>
+      <c r="A14" s="18">
+        <v>1.0</v>
+      </c>
       <c r="B14" s="19" t="s">
         <v>23</v>
       </c>
@@ -908,7 +910,7 @@
     </row>
     <row r="15" ht="24.75" customHeight="1">
       <c r="A15" s="18">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>24</v>
@@ -927,7 +929,7 @@
     </row>
     <row r="16" ht="24.75" customHeight="1">
       <c r="A16" s="18">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>25</v>
@@ -946,7 +948,7 @@
     </row>
     <row r="17" ht="24.75" customHeight="1">
       <c r="A17" s="18">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>26</v>
@@ -965,7 +967,7 @@
     </row>
     <row r="18" ht="24.75" customHeight="1">
       <c r="A18" s="18">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>27</v>
@@ -984,7 +986,7 @@
     </row>
     <row r="19" ht="24.75" customHeight="1">
       <c r="A19" s="18">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>28</v>
@@ -1003,7 +1005,7 @@
     </row>
     <row r="20" ht="24.75" customHeight="1">
       <c r="A20" s="18">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="B20" s="8" t="s">
         <v>29</v>

</xml_diff>